<commit_message>
Update VAT ledger reporting logic and agent metadata
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/POS-Gostinstvo-racunovodski-sledljiv-inventar.xlsx
+++ b/docs/POS-Gostinstvo-racunovodski-sledljiv-inventar.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="691">
   <si>
     <t>POS Gostinstvo — sledljiv inventar računovodskega priročnika</t>
   </si>
@@ -2196,6 +2196,170 @@
   </si>
   <si>
     <t>Priročnik pravilno pokriva dnevni, mesečni in neuspešni prenos ter varno ponavljanje; omejitev je, da je ponovitev dovoljena samo ob dokazani idempotentnosti.</t>
+  </si>
+  <si>
+    <t>TAX-KIR-001</t>
+  </si>
+  <si>
+    <t>davčne evidence</t>
+  </si>
+  <si>
+    <t>KIR – knjiga izdanih računov</t>
+  </si>
+  <si>
+    <t>računovodja
+administrator</t>
+  </si>
+  <si>
+    <t>zaključen POS račun
+veljavna DDV-preslikava</t>
+  </si>
+  <si>
+    <t>Zaključen račun, storno ali vračilo se poveže z vrstico KIR in temeljnico; preverijo se datum, DDV-koda, osnova, DDV, bruto znesek in status.</t>
+  </si>
+  <si>
+    <t>Odprta miza ali manjkajoča preslikava ni KIR; pred izvozom se napaka prikaže in postopek zadrži.</t>
+  </si>
+  <si>
+    <t>Izdani računi in popravki so sledljivi od POS vira do KIR in glavne knjige.</t>
+  </si>
+  <si>
+    <t>artifacts/erp-web/src/pages/ddv-evidence.tsx:101-190</t>
+  </si>
+  <si>
+    <t>artifacts/api-server/src/lib/vatLedger.ts:300-328
+artifacts/api-server/src/lib/vatXmlGenerator.ts:220-244</t>
+  </si>
+  <si>
+    <t>docs/pos-accounting-manual-src/02-prodaja-placila-temeljnice.md:606-619</t>
+  </si>
+  <si>
+    <t>KIR je podprt za pravilno knjižene izdane račune; manjkajoče preslikave blokira predoddajna kontrola.</t>
+  </si>
+  <si>
+    <t>TAX-KPR-001</t>
+  </si>
+  <si>
+    <t>KPR – knjiga prejetih računov</t>
+  </si>
+  <si>
+    <t>potrjen prejeti RACUN
+datum prejema
+veljavna KPR-preslikava</t>
+  </si>
+  <si>
+    <t>Potrjen prejeti račun ustvari KPR-vrstico in vhodno DDV-vrstico; preverijo se dobavitelj, številka, datum listine, datum prejema, DDV, odbitnost in povezava na temeljnico.</t>
+  </si>
+  <si>
+    <t>Prejemnica brez računa ni popoln KPR; manjkajoč datum, koda ali preslikava blokira izvoz.</t>
+  </si>
+  <si>
+    <t>Prejeti računi so vključeni v KPR in povezani z obveznostjo, DDV ter GL.</t>
+  </si>
+  <si>
+    <t>artifacts/erp-web/src/pages/ddv-evidence.tsx:200-290</t>
+  </si>
+  <si>
+    <t>artifacts/api-server/src/lib/vatLedger.ts:209-215
+artifacts/api-server/src/lib/vatXmlGenerator.ts:229-245</t>
+  </si>
+  <si>
+    <t>docs/pos-accounting-manual-src/03-nabava-zaloga-drugi-dogodki.md:801-826</t>
+  </si>
+  <si>
+    <t>KPR je podprt za pravilno knjižene prejete račune; dobropisi/bremepisi sledijo omejitvam svoje knjižne poti.</t>
+  </si>
+  <si>
+    <t>TAX-GL-001</t>
+  </si>
+  <si>
+    <t>Uskladitev KIR/KPR z glavno knjigo</t>
+  </si>
+  <si>
+    <t>zaključeno obdobje
+KIR in KPR pregled
+GL izpis</t>
+  </si>
+  <si>
+    <t>Ročno primerjajte število dokumentov in vrstic, osnove ter DDV po stopnjah, preskoke, dvojnike in korekcijske verige med KIR, KPR in GL.</t>
+  </si>
+  <si>
+    <t>Popoln avtomatski tie-out vseh POS, registrov, banke in GL ni potrjen; razliko zadržite in raziščite po izvorni referenci.</t>
+  </si>
+  <si>
+    <t>Dokumentirana ročna uskladitev zmanjša tveganje manjkajočih ali podvojenih davčnih zapisov.</t>
+  </si>
+  <si>
+    <t>artifacts/erp-web/src/pages/ddv-evidence.tsx:310-350</t>
+  </si>
+  <si>
+    <t>artifacts/api-server/src/routes/vatLedgerReport.ts:206-291</t>
+  </si>
+  <si>
+    <t>docs/pos-accounting-manual-src/00-uvod-in-delo-s-temeljnicami.md:398-404</t>
+  </si>
+  <si>
+    <t>KIR/KPR poročila in kontrole obstajajo, vendar avtomatska popolna uskladitev registra z vsemi viri ni potrjena.</t>
+  </si>
+  <si>
+    <t>TAX-XML-001</t>
+  </si>
+  <si>
+    <t>KIRKPR XML izvoz</t>
+  </si>
+  <si>
+    <t>izbrano podjetje in obdobje
+KIR/KPR brez predoddajnih napak</t>
+  </si>
+  <si>
+    <t>Za izbrano obdobje se preverijo formalne kontrole in preslikave, nato se ustvari ter prenese KIR/KPR XML z rezultatom in številom vrstic.</t>
+  </si>
+  <si>
+    <t>HTTP 422 z razlogi ustavi izvoz ob manjkajoči preslikavi, vatCodeId ali aktivni evidenčni vrstici; delne datoteke ne uporabljajte.</t>
+  </si>
+  <si>
+    <t>Računovodja dobi strojno berljivo datoteko za zunanji postopek oddaje.</t>
+  </si>
+  <si>
+    <t>artifacts/erp-web/src/pages/ddv-evidence.tsx:713-745</t>
+  </si>
+  <si>
+    <t>artifacts/api-server/src/routes/vatSubmissions.ts:180-220
+artifacts/api-server/src/lib/vatXmlGenerator.ts:265-299</t>
+  </si>
+  <si>
+    <t>docs/pos-accounting-manual-src/00-uvod-in-delo-s-temeljnicami.md:406-418</t>
+  </si>
+  <si>
+    <t>XML generiranje in prenos sta implementirana; XML sam po sebi ni dokaz oddaje v eDavke.</t>
+  </si>
+  <si>
+    <t>TAX-EDAVKI-001</t>
+  </si>
+  <si>
+    <t>Neposredna elektronska oddaja KIRKPR v eDavke</t>
+  </si>
+  <si>
+    <t>ustvarjen in preverjen XML
+zunanji odobreni postopek eDavki</t>
+  </si>
+  <si>
+    <t>XML prenesite v zunanji odobreni postopek eDavki in shranite povratnico oziroma zavrnitev skupaj z XML.</t>
+  </si>
+  <si>
+    <t>Aplikacija ne sme prikazati uspešne oddaje brez zunanjega dokazila; napako rešujte z novo preverjeno datoteko.</t>
+  </si>
+  <si>
+    <t>Ločitev priprave XML od dejanske oddaje prepreči lažen dokaz davčne skladnosti.</t>
+  </si>
+  <si>
+    <t>artifacts/api-server/src/routes/vatSubmissions.ts:150-180</t>
+  </si>
+  <si>
+    <t>docs/pos-accounting-manual-src/00-uvod-in-delo-s-temeljnicami.md:420-425</t>
+  </si>
+  <si>
+    <t>Neposredna oddaja iz aplikacije v eDavke ni implementirana; podprt je XML prenos za zunanji postopek.</t>
   </si>
   <si>
     <t>Pokritost</t>
@@ -2519,7 +2683,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>53</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2612,8 +2776,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SledljivInventar" displayName="SledljivInventar" ref="A1:P54" totalsRowShown="0">
-  <autoFilter ref="A1:P54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SledljivInventar" displayName="SledljivInventar" ref="A1:P59" totalsRowShown="0">
+  <autoFilter ref="A1:P59"/>
   <tableColumns count="16">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Področje"/>
@@ -2950,7 +3114,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -2966,7 +3130,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -2996,13 +3160,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="8">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="8">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -3016,7 +3180,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="8">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -3086,7 +3250,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -5803,8 +5967,258 @@
         <v>48</v>
       </c>
     </row>
+    <row r="55" spans="1:16" ht="84" customHeight="1">
+      <c r="A55" s="8" t="s">
+        <v>621</v>
+      </c>
+      <c r="B55" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>623</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="H55" s="7" t="s">
+        <v>628</v>
+      </c>
+      <c r="I55" s="7" t="s">
+        <v>629</v>
+      </c>
+      <c r="J55" s="7" t="s">
+        <v>630</v>
+      </c>
+      <c r="K55" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="L55" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="M55" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N55" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="O55" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="P55" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" ht="84" customHeight="1">
+      <c r="A56" s="8" t="s">
+        <v>633</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>635</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>636</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>637</v>
+      </c>
+      <c r="H56" s="7" t="s">
+        <v>638</v>
+      </c>
+      <c r="I56" s="7" t="s">
+        <v>639</v>
+      </c>
+      <c r="J56" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="K56" s="7" t="s">
+        <v>641</v>
+      </c>
+      <c r="L56" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="M56" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N56" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="O56" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="P56" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="57" spans="1:16" ht="84" customHeight="1">
+      <c r="A57" s="8" t="s">
+        <v>643</v>
+      </c>
+      <c r="B57" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>644</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>645</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="H57" s="7" t="s">
+        <v>648</v>
+      </c>
+      <c r="I57" s="7" t="s">
+        <v>649</v>
+      </c>
+      <c r="J57" s="7" t="s">
+        <v>650</v>
+      </c>
+      <c r="K57" s="7" t="s">
+        <v>651</v>
+      </c>
+      <c r="L57" s="8" t="s">
+        <v>171</v>
+      </c>
+      <c r="M57" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N57" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="O57" s="7" t="s">
+        <v>652</v>
+      </c>
+      <c r="P57" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:16" ht="84" customHeight="1">
+      <c r="A58" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="B58" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>654</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>655</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>656</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>657</v>
+      </c>
+      <c r="H58" s="7" t="s">
+        <v>658</v>
+      </c>
+      <c r="I58" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="J58" s="7" t="s">
+        <v>660</v>
+      </c>
+      <c r="K58" s="7" t="s">
+        <v>661</v>
+      </c>
+      <c r="L58" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="M58" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N58" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="O58" s="7" t="s">
+        <v>662</v>
+      </c>
+      <c r="P58" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="59" spans="1:16" ht="84" customHeight="1">
+      <c r="A59" s="8" t="s">
+        <v>663</v>
+      </c>
+      <c r="B59" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>664</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>665</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>666</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>667</v>
+      </c>
+      <c r="H59" s="7" t="s">
+        <v>668</v>
+      </c>
+      <c r="I59" s="7" t="s">
+        <v>659</v>
+      </c>
+      <c r="J59" s="7" t="s">
+        <v>669</v>
+      </c>
+      <c r="K59" s="7" t="s">
+        <v>670</v>
+      </c>
+      <c r="L59" s="8" t="s">
+        <v>433</v>
+      </c>
+      <c r="M59" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="N59" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="O59" s="7" t="s">
+        <v>671</v>
+      </c>
+      <c r="P59" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="M2:M54">
+  <conditionalFormatting sqref="M2:M59">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PRAVILNO">
       <formula>NOT(ISERROR(SEARCH("PRAVILNO",M2)))</formula>
     </cfRule>
@@ -5818,7 +6232,7 @@
       <formula>NOT(ISERROR(SEARCH("NAPAČNO",M2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N54">
+  <conditionalFormatting sqref="N2:N59">
     <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="KRITIČNO">
       <formula>NOT(ISERROR(SEARCH("KRITIČNO",N2)))</formula>
     </cfRule>
@@ -5855,19 +6269,19 @@
         <v>13</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>621</v>
+        <v>672</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>622</v>
+        <v>673</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>623</v>
+        <v>674</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>624</v>
+        <v>675</v>
       </c>
     </row>
   </sheetData>
@@ -5887,7 +6301,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>625</v>
+        <v>676</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -5895,7 +6309,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>626</v>
+        <v>677</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -5903,7 +6317,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>627</v>
+        <v>678</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -5911,7 +6325,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>628</v>
+        <v>679</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -5919,7 +6333,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>629</v>
+        <v>680</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -5927,7 +6341,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>630</v>
+        <v>681</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -5935,7 +6349,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>626</v>
+        <v>677</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -5943,7 +6357,7 @@
         <v>46</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>631</v>
+        <v>682</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -5951,7 +6365,7 @@
         <v>433</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>632</v>
+        <v>683</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -5959,7 +6373,7 @@
         <v>171</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>633</v>
+        <v>684</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -5967,7 +6381,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>626</v>
+        <v>677</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -5975,7 +6389,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>634</v>
+        <v>685</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -5983,7 +6397,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>635</v>
+        <v>686</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -5991,7 +6405,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>636</v>
+        <v>687</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -5999,17 +6413,17 @@
         <v>18</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>637</v>
+        <v>688</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="3" t="s">
-        <v>638</v>
+        <v>689</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
-        <v>639</v>
+        <v>690</v>
       </c>
       <c r="B21" s="9"/>
     </row>

</xml_diff>

<commit_message>
Update agent memory and documentation assets
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/docs/POS-Gostinstvo-racunovodski-sledljiv-inventar.xlsx
+++ b/docs/POS-Gostinstvo-racunovodski-sledljiv-inventar.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="640">
   <si>
     <t>POS Gostinstvo — sledljiv inventar računovodskega priročnika</t>
   </si>
   <si>
-    <t>Pregled uporabniških postopkov in pokritosti priročnika · 21.09.2026</t>
+    <t>Izvoz inventarja postopkov in pokritosti priročnika · 10.10.2026</t>
   </si>
   <si>
     <t>Osnovni podatki</t>
@@ -2196,170 +2196,6 @@
   </si>
   <si>
     <t>Priročnik pravilno pokriva dnevni, mesečni in neuspešni prenos ter varno ponavljanje; omejitev je, da je ponovitev dovoljena samo ob dokazani idempotentnosti.</t>
-  </si>
-  <si>
-    <t>TAX-KIR-001</t>
-  </si>
-  <si>
-    <t>davčne evidence</t>
-  </si>
-  <si>
-    <t>KIR – knjiga izdanih računov</t>
-  </si>
-  <si>
-    <t>računovodja
-administrator</t>
-  </si>
-  <si>
-    <t>zaključen POS račun
-veljavna DDV-preslikava</t>
-  </si>
-  <si>
-    <t>Zaključen račun, storno ali vračilo se poveže z vrstico KIR in temeljnico; preverijo se datum, DDV-koda, osnova, DDV, bruto znesek in status.</t>
-  </si>
-  <si>
-    <t>Odprta miza ali manjkajoča preslikava ni KIR; pred izvozom se napaka prikaže in postopek zadrži.</t>
-  </si>
-  <si>
-    <t>Izdani računi in popravki so sledljivi od POS vira do KIR in glavne knjige.</t>
-  </si>
-  <si>
-    <t>artifacts/erp-web/src/pages/ddv-evidence.tsx:101-190</t>
-  </si>
-  <si>
-    <t>artifacts/api-server/src/lib/vatLedger.ts:300-328
-artifacts/api-server/src/lib/vatXmlGenerator.ts:220-244</t>
-  </si>
-  <si>
-    <t>docs/pos-accounting-manual-src/02-prodaja-placila-temeljnice.md:606-619</t>
-  </si>
-  <si>
-    <t>KIR je podprt za pravilno knjižene izdane račune; manjkajoče preslikave blokira predoddajna kontrola.</t>
-  </si>
-  <si>
-    <t>TAX-KPR-001</t>
-  </si>
-  <si>
-    <t>KPR – knjiga prejetih računov</t>
-  </si>
-  <si>
-    <t>potrjen prejeti RACUN
-datum prejema
-veljavna KPR-preslikava</t>
-  </si>
-  <si>
-    <t>Potrjen prejeti račun ustvari KPR-vrstico in vhodno DDV-vrstico; preverijo se dobavitelj, številka, datum listine, datum prejema, DDV, odbitnost in povezava na temeljnico.</t>
-  </si>
-  <si>
-    <t>Prejemnica brez računa ni popoln KPR; manjkajoč datum, koda ali preslikava blokira izvoz.</t>
-  </si>
-  <si>
-    <t>Prejeti računi so vključeni v KPR in povezani z obveznostjo, DDV ter GL.</t>
-  </si>
-  <si>
-    <t>artifacts/erp-web/src/pages/ddv-evidence.tsx:200-290</t>
-  </si>
-  <si>
-    <t>artifacts/api-server/src/lib/vatLedger.ts:209-215
-artifacts/api-server/src/lib/vatXmlGenerator.ts:229-245</t>
-  </si>
-  <si>
-    <t>docs/pos-accounting-manual-src/03-nabava-zaloga-drugi-dogodki.md:801-826</t>
-  </si>
-  <si>
-    <t>KPR je podprt za pravilno knjižene prejete račune; dobropisi/bremepisi sledijo omejitvam svoje knjižne poti.</t>
-  </si>
-  <si>
-    <t>TAX-GL-001</t>
-  </si>
-  <si>
-    <t>Uskladitev KIR/KPR z glavno knjigo</t>
-  </si>
-  <si>
-    <t>zaključeno obdobje
-KIR in KPR pregled
-GL izpis</t>
-  </si>
-  <si>
-    <t>Ročno primerjajte število dokumentov in vrstic, osnove ter DDV po stopnjah, preskoke, dvojnike in korekcijske verige med KIR, KPR in GL.</t>
-  </si>
-  <si>
-    <t>Popoln avtomatski tie-out vseh POS, registrov, banke in GL ni potrjen; razliko zadržite in raziščite po izvorni referenci.</t>
-  </si>
-  <si>
-    <t>Dokumentirana ročna uskladitev zmanjša tveganje manjkajočih ali podvojenih davčnih zapisov.</t>
-  </si>
-  <si>
-    <t>artifacts/erp-web/src/pages/ddv-evidence.tsx:310-350</t>
-  </si>
-  <si>
-    <t>artifacts/api-server/src/routes/vatLedgerReport.ts:206-291</t>
-  </si>
-  <si>
-    <t>docs/pos-accounting-manual-src/00-uvod-in-delo-s-temeljnicami.md:398-404</t>
-  </si>
-  <si>
-    <t>KIR/KPR poročila in kontrole obstajajo, vendar avtomatska popolna uskladitev registra z vsemi viri ni potrjena.</t>
-  </si>
-  <si>
-    <t>TAX-XML-001</t>
-  </si>
-  <si>
-    <t>KIRKPR XML izvoz</t>
-  </si>
-  <si>
-    <t>izbrano podjetje in obdobje
-KIR/KPR brez predoddajnih napak</t>
-  </si>
-  <si>
-    <t>Za izbrano obdobje se preverijo formalne kontrole in preslikave, nato se ustvari ter prenese KIR/KPR XML z rezultatom in številom vrstic.</t>
-  </si>
-  <si>
-    <t>HTTP 422 z razlogi ustavi izvoz ob manjkajoči preslikavi, vatCodeId ali aktivni evidenčni vrstici; delne datoteke ne uporabljajte.</t>
-  </si>
-  <si>
-    <t>Računovodja dobi strojno berljivo datoteko za zunanji postopek oddaje.</t>
-  </si>
-  <si>
-    <t>artifacts/erp-web/src/pages/ddv-evidence.tsx:713-745</t>
-  </si>
-  <si>
-    <t>artifacts/api-server/src/routes/vatSubmissions.ts:180-220
-artifacts/api-server/src/lib/vatXmlGenerator.ts:265-299</t>
-  </si>
-  <si>
-    <t>docs/pos-accounting-manual-src/00-uvod-in-delo-s-temeljnicami.md:406-418</t>
-  </si>
-  <si>
-    <t>XML generiranje in prenos sta implementirana; XML sam po sebi ni dokaz oddaje v eDavke.</t>
-  </si>
-  <si>
-    <t>TAX-EDAVKI-001</t>
-  </si>
-  <si>
-    <t>Neposredna elektronska oddaja KIRKPR v eDavke</t>
-  </si>
-  <si>
-    <t>ustvarjen in preverjen XML
-zunanji odobreni postopek eDavki</t>
-  </si>
-  <si>
-    <t>XML prenesite v zunanji odobreni postopek eDavki in shranite povratnico oziroma zavrnitev skupaj z XML.</t>
-  </si>
-  <si>
-    <t>Aplikacija ne sme prikazati uspešne oddaje brez zunanjega dokazila; napako rešujte z novo preverjeno datoteko.</t>
-  </si>
-  <si>
-    <t>Ločitev priprave XML od dejanske oddaje prepreči lažen dokaz davčne skladnosti.</t>
-  </si>
-  <si>
-    <t>artifacts/api-server/src/routes/vatSubmissions.ts:150-180</t>
-  </si>
-  <si>
-    <t>docs/pos-accounting-manual-src/00-uvod-in-delo-s-temeljnicami.md:420-425</t>
-  </si>
-  <si>
-    <t>Neposredna oddaja iz aplikacije v eDavke ni implementirana; podprt je XML prenos za zunanji postopek.</t>
   </si>
   <si>
     <t>Pokritost</t>
@@ -2683,7 +2519,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>58</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2776,8 +2612,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SledljivInventar" displayName="SledljivInventar" ref="A1:P59" totalsRowShown="0">
-  <autoFilter ref="A1:P59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SledljivInventar" displayName="SledljivInventar" ref="A1:P54" totalsRowShown="0">
+  <autoFilter ref="A1:P54"/>
   <tableColumns count="16">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Področje"/>
@@ -3114,7 +2950,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="5">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -3130,7 +2966,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -3160,13 +2996,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="8">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>15</v>
       </c>
       <c r="E11" s="8">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -3180,7 +3016,7 @@
         <v>16</v>
       </c>
       <c r="E12" s="8">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -3250,7 +3086,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P59"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -5967,258 +5803,8 @@
         <v>48</v>
       </c>
     </row>
-    <row r="55" spans="1:16" ht="84" customHeight="1">
-      <c r="A55" s="8" t="s">
-        <v>621</v>
-      </c>
-      <c r="B55" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="C55" s="7" t="s">
-        <v>623</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>624</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>625</v>
-      </c>
-      <c r="F55" s="7" t="s">
-        <v>626</v>
-      </c>
-      <c r="G55" s="7" t="s">
-        <v>627</v>
-      </c>
-      <c r="H55" s="7" t="s">
-        <v>628</v>
-      </c>
-      <c r="I55" s="7" t="s">
-        <v>629</v>
-      </c>
-      <c r="J55" s="7" t="s">
-        <v>630</v>
-      </c>
-      <c r="K55" s="7" t="s">
-        <v>631</v>
-      </c>
-      <c r="L55" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="M55" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="N55" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="O55" s="7" t="s">
-        <v>632</v>
-      </c>
-      <c r="P55" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" ht="84" customHeight="1">
-      <c r="A56" s="8" t="s">
-        <v>633</v>
-      </c>
-      <c r="B56" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>634</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>624</v>
-      </c>
-      <c r="E56" s="7" t="s">
-        <v>635</v>
-      </c>
-      <c r="F56" s="7" t="s">
-        <v>636</v>
-      </c>
-      <c r="G56" s="7" t="s">
-        <v>637</v>
-      </c>
-      <c r="H56" s="7" t="s">
-        <v>638</v>
-      </c>
-      <c r="I56" s="7" t="s">
-        <v>639</v>
-      </c>
-      <c r="J56" s="7" t="s">
-        <v>640</v>
-      </c>
-      <c r="K56" s="7" t="s">
-        <v>641</v>
-      </c>
-      <c r="L56" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="M56" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="N56" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="O56" s="7" t="s">
-        <v>642</v>
-      </c>
-      <c r="P56" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="57" spans="1:16" ht="84" customHeight="1">
-      <c r="A57" s="8" t="s">
-        <v>643</v>
-      </c>
-      <c r="B57" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>644</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="E57" s="7" t="s">
-        <v>645</v>
-      </c>
-      <c r="F57" s="7" t="s">
-        <v>646</v>
-      </c>
-      <c r="G57" s="7" t="s">
-        <v>647</v>
-      </c>
-      <c r="H57" s="7" t="s">
-        <v>648</v>
-      </c>
-      <c r="I57" s="7" t="s">
-        <v>649</v>
-      </c>
-      <c r="J57" s="7" t="s">
-        <v>650</v>
-      </c>
-      <c r="K57" s="7" t="s">
-        <v>651</v>
-      </c>
-      <c r="L57" s="8" t="s">
-        <v>171</v>
-      </c>
-      <c r="M57" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="N57" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="O57" s="7" t="s">
-        <v>652</v>
-      </c>
-      <c r="P57" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="58" spans="1:16" ht="84" customHeight="1">
-      <c r="A58" s="8" t="s">
-        <v>653</v>
-      </c>
-      <c r="B58" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="C58" s="7" t="s">
-        <v>654</v>
-      </c>
-      <c r="D58" s="7" t="s">
-        <v>624</v>
-      </c>
-      <c r="E58" s="7" t="s">
-        <v>655</v>
-      </c>
-      <c r="F58" s="7" t="s">
-        <v>656</v>
-      </c>
-      <c r="G58" s="7" t="s">
-        <v>657</v>
-      </c>
-      <c r="H58" s="7" t="s">
-        <v>658</v>
-      </c>
-      <c r="I58" s="7" t="s">
-        <v>659</v>
-      </c>
-      <c r="J58" s="7" t="s">
-        <v>660</v>
-      </c>
-      <c r="K58" s="7" t="s">
-        <v>661</v>
-      </c>
-      <c r="L58" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="M58" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="N58" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="O58" s="7" t="s">
-        <v>662</v>
-      </c>
-      <c r="P58" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="59" spans="1:16" ht="84" customHeight="1">
-      <c r="A59" s="8" t="s">
-        <v>663</v>
-      </c>
-      <c r="B59" s="7" t="s">
-        <v>622</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>664</v>
-      </c>
-      <c r="D59" s="7" t="s">
-        <v>624</v>
-      </c>
-      <c r="E59" s="7" t="s">
-        <v>665</v>
-      </c>
-      <c r="F59" s="7" t="s">
-        <v>666</v>
-      </c>
-      <c r="G59" s="7" t="s">
-        <v>667</v>
-      </c>
-      <c r="H59" s="7" t="s">
-        <v>668</v>
-      </c>
-      <c r="I59" s="7" t="s">
-        <v>659</v>
-      </c>
-      <c r="J59" s="7" t="s">
-        <v>669</v>
-      </c>
-      <c r="K59" s="7" t="s">
-        <v>670</v>
-      </c>
-      <c r="L59" s="8" t="s">
-        <v>433</v>
-      </c>
-      <c r="M59" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="N59" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="O59" s="7" t="s">
-        <v>671</v>
-      </c>
-      <c r="P59" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="M2:M59">
+  <conditionalFormatting sqref="M2:M54">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="PRAVILNO">
       <formula>NOT(ISERROR(SEARCH("PRAVILNO",M2)))</formula>
     </cfRule>
@@ -6232,7 +5818,7 @@
       <formula>NOT(ISERROR(SEARCH("NAPAČNO",M2)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N59">
+  <conditionalFormatting sqref="N2:N54">
     <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="KRITIČNO">
       <formula>NOT(ISERROR(SEARCH("KRITIČNO",N2)))</formula>
     </cfRule>
@@ -6269,19 +5855,19 @@
         <v>13</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>672</v>
+        <v>621</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>22</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>673</v>
+        <v>622</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>674</v>
+        <v>623</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>675</v>
+        <v>624</v>
       </c>
     </row>
   </sheetData>
@@ -6301,7 +5887,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>676</v>
+        <v>625</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -6309,7 +5895,7 @@
         <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>677</v>
+        <v>626</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -6317,7 +5903,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>678</v>
+        <v>627</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -6325,7 +5911,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>679</v>
+        <v>628</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -6333,7 +5919,7 @@
         <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>680</v>
+        <v>629</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -6341,7 +5927,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>681</v>
+        <v>630</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -6349,7 +5935,7 @@
         <v>32</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>677</v>
+        <v>626</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -6357,7 +5943,7 @@
         <v>46</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>682</v>
+        <v>631</v>
       </c>
     </row>
     <row r="11" spans="1:2">
@@ -6365,7 +5951,7 @@
         <v>433</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>683</v>
+        <v>632</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -6373,7 +5959,7 @@
         <v>171</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>684</v>
+        <v>633</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -6381,7 +5967,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>677</v>
+        <v>626</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -6389,7 +5975,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>685</v>
+        <v>634</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -6397,7 +5983,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>686</v>
+        <v>635</v>
       </c>
     </row>
     <row r="17" spans="1:2">
@@ -6405,7 +5991,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>687</v>
+        <v>636</v>
       </c>
     </row>
     <row r="18" spans="1:2">
@@ -6413,17 +5999,17 @@
         <v>18</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>688</v>
+        <v>637</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20" s="3" t="s">
-        <v>689</v>
+        <v>638</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21" s="9" t="s">
-        <v>690</v>
+        <v>639</v>
       </c>
       <c r="B21" s="9"/>
     </row>

</xml_diff>